<commit_message>
Thêm nhật ký sử dụng gói DV v2
</commit_message>
<xml_diff>
--- a/banhang24/Template/ExportExcel/Report/BaoCaoGoiDichVu/Teamplate_TonDichVuChuaSuDung.xlsx
+++ b/banhang24/Template/ExportExcel/Report/BaoCaoGoiDichVu/Teamplate_TonDichVuChuaSuDung.xlsx
@@ -17,10 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>Tổng cộng:</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Số lượng bán</t>
   </si>
@@ -108,7 +105,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -120,14 +117,8 @@
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -150,49 +141,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -216,9 +170,6 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -236,15 +187,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -551,10 +493,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" style="12" customWidth="1"/>
+    <col min="1" max="1" width="20" style="11" customWidth="1"/>
     <col min="2" max="2" width="34.28515625" style="5" customWidth="1"/>
     <col min="3" max="3" width="21.140625" style="5" customWidth="1"/>
     <col min="4" max="4" width="22.5703125" style="5" customWidth="1"/>
@@ -567,77 +509,77 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="3"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+    </row>
+    <row r="4" spans="1:13" s="6" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="3"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:13" s="6" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="11" t="s">
+      <c r="G4" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="J4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="I4" s="11" t="s">
+      <c r="K4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="L4" s="10" t="s">
         <v>8</v>
-      </c>
-      <c r="K4" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -976,51 +918,10 @@
       <c r="K28" s="7"/>
       <c r="L28" s="7"/>
     </row>
-    <row r="29" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="9">
-        <f>SUM(E$5:E28)</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="9">
-        <f>SUM(F$5:F28)</f>
-        <v>0</v>
-      </c>
-      <c r="G29" s="9">
-        <f>SUM(G$5:G28)</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="9">
-        <f>SUM(H$5:H28)</f>
-        <v>0</v>
-      </c>
-      <c r="I29" s="9">
-        <f>SUM(I$5:I28)</f>
-        <v>0</v>
-      </c>
-      <c r="J29" s="9">
-        <f>SUM(J$5:J28)</f>
-        <v>0</v>
-      </c>
-      <c r="K29" s="9">
-        <f>SUM(K$5:K28)</f>
-        <v>0</v>
-      </c>
-      <c r="L29" s="9">
-        <f>SUM(L$5:L28)</f>
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A29:D29"/>
   </mergeCells>
   <pageMargins left="0.76" right="0.23" top="0.78" bottom="0.87" header="0.3" footer="0.7"/>
   <pageSetup scale="95" orientation="landscape" r:id="rId1"/>

</xml_diff>